<commit_message>
Update README and add evaluation and prompt resources.
</commit_message>
<xml_diff>
--- a/resources/evaluation/mSEC-AT_calculations_times.xlsx
+++ b/resources/evaluation/mSEC-AT_calculations_times.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjlop\Proyectos\mSEC-AT\resources\evaluation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjlop\Universidad\doctorado\Trabajo 13 mSEC-AT\envio\revision1\finales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{600D6AE4-80CD-457A-84D0-AAE9EAC94EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569DF761-02FC-42A8-8735-670685C9CA60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CA4F6415-5AB0-4CFD-9911-8D03A96E2097}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CA4F6415-5AB0-4CFD-9911-8D03A96E2097}"/>
   </bookViews>
   <sheets>
     <sheet name="Datas" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="131">
   <si>
     <t>Signal Android</t>
   </si>
@@ -457,6 +457,9 @@
   </si>
   <si>
     <t>Testing repository</t>
+  </si>
+  <si>
+    <t>3.1.1</t>
   </si>
 </sst>
 </file>
@@ -1642,7 +1645,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A2740497-1ACF-40FD-8E36-39E40EE32161}" type="CELLRANGE">
+                    <a:fld id="{214D265F-5184-4229-A01C-73B46E9289BF}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5403,165 +5406,165 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D311EADF-B027-440D-BD0E-A6D20B2AC162}">
   <dimension ref="A1:FN12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" customWidth="1"/>
-    <col min="3" max="3" width="65.109375" customWidth="1"/>
-    <col min="4" max="4" width="52.5546875" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" customWidth="1"/>
-    <col min="6" max="6" width="69.88671875" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.6640625" customWidth="1"/>
-    <col min="9" max="10" width="19.44140625" customWidth="1"/>
-    <col min="11" max="11" width="18.44140625" customWidth="1"/>
-    <col min="12" max="12" width="12.44140625" customWidth="1"/>
-    <col min="13" max="13" width="16.33203125" customWidth="1"/>
-    <col min="14" max="14" width="19.5546875" customWidth="1"/>
-    <col min="15" max="15" width="17.6640625" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="65.140625" customWidth="1"/>
+    <col min="4" max="4" width="52.5703125" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" customWidth="1"/>
+    <col min="6" max="6" width="69.85546875" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" customWidth="1"/>
+    <col min="9" max="10" width="19.42578125" customWidth="1"/>
+    <col min="11" max="11" width="18.42578125" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" customWidth="1"/>
+    <col min="13" max="13" width="16.28515625" customWidth="1"/>
+    <col min="14" max="14" width="19.5703125" customWidth="1"/>
+    <col min="15" max="15" width="17.7109375" customWidth="1"/>
     <col min="16" max="16" width="25" customWidth="1"/>
-    <col min="17" max="17" width="21.5546875" customWidth="1"/>
-    <col min="18" max="18" width="27.33203125" customWidth="1"/>
-    <col min="19" max="19" width="30.6640625" customWidth="1"/>
-    <col min="20" max="20" width="14.88671875" customWidth="1"/>
-    <col min="21" max="21" width="16.33203125" customWidth="1"/>
+    <col min="17" max="17" width="21.5703125" customWidth="1"/>
+    <col min="18" max="18" width="27.28515625" customWidth="1"/>
+    <col min="19" max="19" width="30.7109375" customWidth="1"/>
+    <col min="20" max="20" width="14.85546875" customWidth="1"/>
+    <col min="21" max="21" width="16.28515625" customWidth="1"/>
     <col min="22" max="22" width="17" customWidth="1"/>
-    <col min="23" max="23" width="23.44140625" customWidth="1"/>
-    <col min="24" max="24" width="18.109375" customWidth="1"/>
-    <col min="25" max="25" width="17.6640625" customWidth="1"/>
+    <col min="23" max="23" width="23.42578125" customWidth="1"/>
+    <col min="24" max="24" width="18.140625" customWidth="1"/>
+    <col min="25" max="25" width="17.7109375" customWidth="1"/>
     <col min="26" max="27" width="22" customWidth="1"/>
     <col min="28" max="29" width="31" customWidth="1"/>
-    <col min="30" max="30" width="30.44140625" customWidth="1"/>
-    <col min="31" max="31" width="33.33203125" customWidth="1"/>
-    <col min="32" max="32" width="27.33203125" customWidth="1"/>
+    <col min="30" max="30" width="30.42578125" customWidth="1"/>
+    <col min="31" max="31" width="33.28515625" customWidth="1"/>
+    <col min="32" max="32" width="27.28515625" customWidth="1"/>
     <col min="33" max="33" width="31" customWidth="1"/>
-    <col min="34" max="34" width="14.109375" customWidth="1"/>
-    <col min="35" max="35" width="16.88671875" customWidth="1"/>
-    <col min="36" max="36" width="19.109375" customWidth="1"/>
-    <col min="37" max="37" width="26.109375" customWidth="1"/>
+    <col min="34" max="34" width="14.140625" customWidth="1"/>
+    <col min="35" max="35" width="16.85546875" customWidth="1"/>
+    <col min="36" max="36" width="19.140625" customWidth="1"/>
+    <col min="37" max="37" width="26.140625" customWidth="1"/>
     <col min="38" max="38" width="19" customWidth="1"/>
-    <col min="39" max="39" width="16.33203125" customWidth="1"/>
-    <col min="40" max="41" width="22.33203125" customWidth="1"/>
-    <col min="42" max="42" width="31.6640625" customWidth="1"/>
+    <col min="39" max="39" width="16.28515625" customWidth="1"/>
+    <col min="40" max="41" width="22.28515625" customWidth="1"/>
+    <col min="42" max="42" width="31.7109375" customWidth="1"/>
     <col min="43" max="43" width="33" customWidth="1"/>
-    <col min="44" max="44" width="30.88671875" customWidth="1"/>
-    <col min="45" max="45" width="33.44140625" customWidth="1"/>
-    <col min="46" max="46" width="25.88671875" customWidth="1"/>
-    <col min="47" max="47" width="31.109375" customWidth="1"/>
-    <col min="48" max="48" width="14.88671875" customWidth="1"/>
-    <col min="49" max="49" width="16.6640625" customWidth="1"/>
-    <col min="50" max="50" width="15.109375" customWidth="1"/>
+    <col min="44" max="44" width="30.85546875" customWidth="1"/>
+    <col min="45" max="45" width="33.42578125" customWidth="1"/>
+    <col min="46" max="46" width="25.85546875" customWidth="1"/>
+    <col min="47" max="47" width="31.140625" customWidth="1"/>
+    <col min="48" max="48" width="14.85546875" customWidth="1"/>
+    <col min="49" max="49" width="16.7109375" customWidth="1"/>
+    <col min="50" max="50" width="15.140625" customWidth="1"/>
     <col min="51" max="51" width="24" customWidth="1"/>
-    <col min="52" max="52" width="17.88671875" customWidth="1"/>
-    <col min="53" max="53" width="17.33203125" customWidth="1"/>
-    <col min="54" max="55" width="23.5546875" customWidth="1"/>
-    <col min="56" max="56" width="31.6640625" customWidth="1"/>
-    <col min="57" max="57" width="33.5546875" customWidth="1"/>
-    <col min="58" max="58" width="32.5546875" customWidth="1"/>
-    <col min="59" max="59" width="33.88671875" customWidth="1"/>
-    <col min="60" max="60" width="28.33203125" customWidth="1"/>
-    <col min="61" max="61" width="28.5546875" customWidth="1"/>
-    <col min="62" max="62" width="14.88671875" customWidth="1"/>
-    <col min="63" max="63" width="17.6640625" customWidth="1"/>
+    <col min="52" max="52" width="17.85546875" customWidth="1"/>
+    <col min="53" max="53" width="17.28515625" customWidth="1"/>
+    <col min="54" max="55" width="23.5703125" customWidth="1"/>
+    <col min="56" max="56" width="31.7109375" customWidth="1"/>
+    <col min="57" max="57" width="33.5703125" customWidth="1"/>
+    <col min="58" max="58" width="32.5703125" customWidth="1"/>
+    <col min="59" max="59" width="33.85546875" customWidth="1"/>
+    <col min="60" max="60" width="28.28515625" customWidth="1"/>
+    <col min="61" max="61" width="28.5703125" customWidth="1"/>
+    <col min="62" max="62" width="14.85546875" customWidth="1"/>
+    <col min="63" max="63" width="17.7109375" customWidth="1"/>
     <col min="64" max="64" width="15" customWidth="1"/>
     <col min="65" max="65" width="25" customWidth="1"/>
-    <col min="66" max="66" width="19.6640625" customWidth="1"/>
-    <col min="67" max="67" width="19.44140625" customWidth="1"/>
-    <col min="68" max="68" width="24.109375" customWidth="1"/>
+    <col min="66" max="66" width="19.7109375" customWidth="1"/>
+    <col min="67" max="67" width="19.42578125" customWidth="1"/>
+    <col min="68" max="68" width="24.140625" customWidth="1"/>
     <col min="69" max="69" width="22" customWidth="1"/>
-    <col min="70" max="70" width="32.6640625" customWidth="1"/>
-    <col min="71" max="72" width="31.6640625" customWidth="1"/>
-    <col min="73" max="73" width="34.33203125" customWidth="1"/>
+    <col min="70" max="70" width="32.7109375" customWidth="1"/>
+    <col min="71" max="72" width="31.7109375" customWidth="1"/>
+    <col min="73" max="73" width="34.28515625" customWidth="1"/>
     <col min="74" max="74" width="26" customWidth="1"/>
-    <col min="75" max="75" width="28.44140625" customWidth="1"/>
-    <col min="76" max="76" width="14.33203125" customWidth="1"/>
-    <col min="77" max="77" width="16.33203125" customWidth="1"/>
-    <col min="78" max="78" width="15.44140625" customWidth="1"/>
-    <col min="79" max="79" width="25.6640625" customWidth="1"/>
-    <col min="80" max="80" width="19.33203125" customWidth="1"/>
+    <col min="75" max="75" width="28.42578125" customWidth="1"/>
+    <col min="76" max="76" width="14.28515625" customWidth="1"/>
+    <col min="77" max="77" width="16.28515625" customWidth="1"/>
+    <col min="78" max="78" width="15.42578125" customWidth="1"/>
+    <col min="79" max="79" width="25.7109375" customWidth="1"/>
+    <col min="80" max="80" width="19.28515625" customWidth="1"/>
     <col min="81" max="81" width="17" customWidth="1"/>
-    <col min="82" max="83" width="24.109375" customWidth="1"/>
+    <col min="82" max="83" width="24.140625" customWidth="1"/>
     <col min="84" max="84" width="34" customWidth="1"/>
-    <col min="85" max="85" width="32.44140625" customWidth="1"/>
-    <col min="86" max="86" width="30.6640625" customWidth="1"/>
-    <col min="87" max="87" width="35.109375" customWidth="1"/>
-    <col min="88" max="88" width="25.33203125" customWidth="1"/>
-    <col min="89" max="89" width="28.6640625" customWidth="1"/>
-    <col min="90" max="90" width="15.6640625" customWidth="1"/>
-    <col min="91" max="91" width="17.109375" customWidth="1"/>
-    <col min="92" max="92" width="15.6640625" customWidth="1"/>
-    <col min="93" max="93" width="24.5546875" customWidth="1"/>
-    <col min="94" max="94" width="17.6640625" customWidth="1"/>
-    <col min="95" max="95" width="15.6640625" customWidth="1"/>
-    <col min="96" max="97" width="23.33203125" customWidth="1"/>
-    <col min="98" max="98" width="31.33203125" customWidth="1"/>
-    <col min="99" max="99" width="34.88671875" customWidth="1"/>
-    <col min="100" max="100" width="32.44140625" customWidth="1"/>
-    <col min="101" max="101" width="34.109375" customWidth="1"/>
-    <col min="102" max="102" width="26.109375" customWidth="1"/>
-    <col min="103" max="103" width="28.6640625" customWidth="1"/>
+    <col min="85" max="85" width="32.42578125" customWidth="1"/>
+    <col min="86" max="86" width="30.7109375" customWidth="1"/>
+    <col min="87" max="87" width="35.140625" customWidth="1"/>
+    <col min="88" max="88" width="25.28515625" customWidth="1"/>
+    <col min="89" max="89" width="28.7109375" customWidth="1"/>
+    <col min="90" max="90" width="15.7109375" customWidth="1"/>
+    <col min="91" max="91" width="17.140625" customWidth="1"/>
+    <col min="92" max="92" width="15.7109375" customWidth="1"/>
+    <col min="93" max="93" width="24.5703125" customWidth="1"/>
+    <col min="94" max="94" width="17.7109375" customWidth="1"/>
+    <col min="95" max="95" width="15.7109375" customWidth="1"/>
+    <col min="96" max="97" width="23.28515625" customWidth="1"/>
+    <col min="98" max="98" width="31.28515625" customWidth="1"/>
+    <col min="99" max="99" width="34.85546875" customWidth="1"/>
+    <col min="100" max="100" width="32.42578125" customWidth="1"/>
+    <col min="101" max="101" width="34.140625" customWidth="1"/>
+    <col min="102" max="102" width="26.140625" customWidth="1"/>
+    <col min="103" max="103" width="28.7109375" customWidth="1"/>
     <col min="104" max="104" width="17" customWidth="1"/>
-    <col min="105" max="105" width="18.33203125" customWidth="1"/>
-    <col min="106" max="106" width="15.33203125" customWidth="1"/>
+    <col min="105" max="105" width="18.28515625" customWidth="1"/>
+    <col min="106" max="106" width="15.28515625" customWidth="1"/>
     <col min="107" max="107" width="24" customWidth="1"/>
-    <col min="108" max="108" width="20.44140625" customWidth="1"/>
-    <col min="109" max="109" width="17.6640625" customWidth="1"/>
-    <col min="110" max="110" width="23.88671875" customWidth="1"/>
-    <col min="111" max="111" width="22.44140625" customWidth="1"/>
-    <col min="112" max="112" width="32.109375" customWidth="1"/>
-    <col min="113" max="113" width="34.44140625" customWidth="1"/>
-    <col min="114" max="114" width="30.5546875" customWidth="1"/>
-    <col min="115" max="115" width="34.5546875" customWidth="1"/>
-    <col min="116" max="116" width="25.6640625" customWidth="1"/>
-    <col min="117" max="117" width="28.5546875" customWidth="1"/>
-    <col min="118" max="118" width="15.5546875" customWidth="1"/>
-    <col min="119" max="119" width="17.33203125" customWidth="1"/>
+    <col min="108" max="108" width="20.42578125" customWidth="1"/>
+    <col min="109" max="109" width="17.7109375" customWidth="1"/>
+    <col min="110" max="110" width="23.85546875" customWidth="1"/>
+    <col min="111" max="111" width="22.42578125" customWidth="1"/>
+    <col min="112" max="112" width="32.140625" customWidth="1"/>
+    <col min="113" max="113" width="34.42578125" customWidth="1"/>
+    <col min="114" max="114" width="30.5703125" customWidth="1"/>
+    <col min="115" max="115" width="34.5703125" customWidth="1"/>
+    <col min="116" max="116" width="25.7109375" customWidth="1"/>
+    <col min="117" max="117" width="28.5703125" customWidth="1"/>
+    <col min="118" max="118" width="15.5703125" customWidth="1"/>
+    <col min="119" max="119" width="17.28515625" customWidth="1"/>
     <col min="120" max="120" width="15" customWidth="1"/>
     <col min="121" max="121" width="25" customWidth="1"/>
-    <col min="122" max="122" width="18.44140625" customWidth="1"/>
-    <col min="123" max="123" width="17.6640625" customWidth="1"/>
-    <col min="124" max="125" width="23.88671875" customWidth="1"/>
+    <col min="122" max="122" width="18.42578125" customWidth="1"/>
+    <col min="123" max="123" width="17.7109375" customWidth="1"/>
+    <col min="124" max="125" width="23.85546875" customWidth="1"/>
     <col min="126" max="126" width="32" customWidth="1"/>
-    <col min="127" max="127" width="30.88671875" customWidth="1"/>
-    <col min="128" max="128" width="30.6640625" customWidth="1"/>
-    <col min="129" max="129" width="34.6640625" customWidth="1"/>
-    <col min="130" max="130" width="27.6640625" customWidth="1"/>
-    <col min="131" max="131" width="28.88671875" customWidth="1"/>
-    <col min="132" max="132" width="17.109375" customWidth="1"/>
-    <col min="133" max="133" width="16.109375" customWidth="1"/>
-    <col min="134" max="134" width="18.33203125" customWidth="1"/>
-    <col min="135" max="135" width="23.6640625" customWidth="1"/>
-    <col min="136" max="136" width="21.5546875" customWidth="1"/>
-    <col min="137" max="137" width="19.33203125" customWidth="1"/>
+    <col min="127" max="127" width="30.85546875" customWidth="1"/>
+    <col min="128" max="128" width="30.7109375" customWidth="1"/>
+    <col min="129" max="129" width="34.7109375" customWidth="1"/>
+    <col min="130" max="130" width="27.7109375" customWidth="1"/>
+    <col min="131" max="131" width="28.85546875" customWidth="1"/>
+    <col min="132" max="132" width="17.140625" customWidth="1"/>
+    <col min="133" max="133" width="16.140625" customWidth="1"/>
+    <col min="134" max="134" width="18.28515625" customWidth="1"/>
+    <col min="135" max="135" width="23.7109375" customWidth="1"/>
+    <col min="136" max="136" width="21.5703125" customWidth="1"/>
+    <col min="137" max="137" width="19.28515625" customWidth="1"/>
     <col min="138" max="139" width="23" customWidth="1"/>
-    <col min="140" max="140" width="29.5546875" customWidth="1"/>
+    <col min="140" max="140" width="29.5703125" customWidth="1"/>
     <col min="141" max="141" width="32" customWidth="1"/>
-    <col min="142" max="142" width="30.44140625" customWidth="1"/>
-    <col min="143" max="143" width="32.109375" customWidth="1"/>
-    <col min="144" max="144" width="26.109375" customWidth="1"/>
-    <col min="145" max="145" width="29.5546875" customWidth="1"/>
-    <col min="146" max="146" width="14.33203125" customWidth="1"/>
-    <col min="147" max="147" width="15.5546875" customWidth="1"/>
-    <col min="148" max="148" width="14.6640625" customWidth="1"/>
-    <col min="149" max="149" width="22.6640625" customWidth="1"/>
-    <col min="150" max="150" width="17.6640625" customWidth="1"/>
-    <col min="151" max="151" width="17.109375" customWidth="1"/>
-    <col min="152" max="153" width="22.88671875" customWidth="1"/>
-    <col min="154" max="154" width="31.6640625" customWidth="1"/>
-    <col min="155" max="155" width="29.6640625" customWidth="1"/>
+    <col min="142" max="142" width="30.42578125" customWidth="1"/>
+    <col min="143" max="143" width="32.140625" customWidth="1"/>
+    <col min="144" max="144" width="26.140625" customWidth="1"/>
+    <col min="145" max="145" width="29.5703125" customWidth="1"/>
+    <col min="146" max="146" width="14.28515625" customWidth="1"/>
+    <col min="147" max="147" width="15.5703125" customWidth="1"/>
+    <col min="148" max="148" width="14.7109375" customWidth="1"/>
+    <col min="149" max="149" width="22.7109375" customWidth="1"/>
+    <col min="150" max="150" width="17.7109375" customWidth="1"/>
+    <col min="151" max="151" width="17.140625" customWidth="1"/>
+    <col min="152" max="153" width="22.85546875" customWidth="1"/>
+    <col min="154" max="154" width="31.7109375" customWidth="1"/>
+    <col min="155" max="155" width="29.7109375" customWidth="1"/>
     <col min="156" max="156" width="29" customWidth="1"/>
-    <col min="157" max="157" width="32.6640625" customWidth="1"/>
+    <col min="157" max="157" width="32.7109375" customWidth="1"/>
     <col min="158" max="158" width="29" customWidth="1"/>
-    <col min="159" max="159" width="28.109375" customWidth="1"/>
-    <col min="160" max="160" width="14.33203125" customWidth="1"/>
-    <col min="161" max="161" width="16.6640625" customWidth="1"/>
-    <col min="162" max="162" width="14.6640625" customWidth="1"/>
-    <col min="163" max="163" width="21.33203125" customWidth="1"/>
+    <col min="159" max="159" width="28.140625" customWidth="1"/>
+    <col min="160" max="160" width="14.28515625" customWidth="1"/>
+    <col min="161" max="161" width="16.7109375" customWidth="1"/>
+    <col min="162" max="162" width="14.7109375" customWidth="1"/>
+    <col min="163" max="163" width="21.28515625" customWidth="1"/>
     <col min="164" max="164" width="16" customWidth="1"/>
     <col min="165" max="165" width="17" customWidth="1"/>
-    <col min="167" max="167" width="14.6640625" customWidth="1"/>
-    <col min="168" max="168" width="15.33203125" customWidth="1"/>
-    <col min="169" max="169" width="13.33203125" customWidth="1"/>
+    <col min="167" max="167" width="14.7109375" customWidth="1"/>
+    <col min="168" max="168" width="15.28515625" customWidth="1"/>
+    <col min="169" max="169" width="13.28515625" customWidth="1"/>
     <col min="170" max="170" width="16" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9598,8 +9601,8 @@
       <c r="A11" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="1">
-        <v>1</v>
+      <c r="B11" s="1" t="s">
+        <v>130</v>
       </c>
       <c r="C11" t="s">
         <v>33</v>
@@ -10217,11 +10220,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FA5DB4D-C211-4325-8C6A-EF547016896B}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="37.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.33203125" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -10497,9 +10500,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3DF7A93-1C1C-411C-8BB4-C1B5023E23E2}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.5546875" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -10591,11 +10594,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6922181F-4CD6-4C05-8D6F-4C0F78BDF1E3}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="38.88671875" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="38.85546875" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -10716,16 +10719,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F64B3DA-5059-482C-8666-A1F90B095773}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="32.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="42.44140625" customWidth="1"/>
-    <col min="4" max="4" width="19.44140625" customWidth="1"/>
-    <col min="5" max="5" width="26.88671875" customWidth="1"/>
+    <col min="1" max="1" width="32.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="42.42578125" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="17.5546875" customWidth="1"/>
-    <col min="9" max="9" width="23.5546875" customWidth="1"/>
+    <col min="7" max="7" width="17.5703125" customWidth="1"/>
+    <col min="9" max="9" width="23.5703125" customWidth="1"/>
     <col min="10" max="10" width="28" customWidth="1"/>
   </cols>
   <sheetData>
@@ -11002,12 +11005,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A52AD7BD-0375-48E7-99C5-DFF4D1DB57B5}">
   <dimension ref="A1:E202"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="35.88671875" customWidth="1"/>
-    <col min="3" max="3" width="18.88671875" customWidth="1"/>
+    <col min="1" max="1" width="35.85546875" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -13367,16 +13370,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A104:E104"/>
+    <mergeCell ref="A125:E125"/>
+    <mergeCell ref="A146:E146"/>
+    <mergeCell ref="A167:E167"/>
+    <mergeCell ref="A188:E188"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A41:E41"/>
     <mergeCell ref="A62:E62"/>
     <mergeCell ref="A83:E83"/>
-    <mergeCell ref="A104:E104"/>
-    <mergeCell ref="A125:E125"/>
-    <mergeCell ref="A146:E146"/>
-    <mergeCell ref="A167:E167"/>
-    <mergeCell ref="A188:E188"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13385,17 +13388,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{198F608C-990B-4493-93E8-88DBB1B15944}">
   <dimension ref="A1:M23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="37.88671875" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" customWidth="1"/>
-    <col min="4" max="4" width="20.109375" customWidth="1"/>
-    <col min="5" max="5" width="17.44140625" customWidth="1"/>
-    <col min="7" max="7" width="24.5546875" customWidth="1"/>
-    <col min="8" max="8" width="25.88671875" customWidth="1"/>
-    <col min="9" max="9" width="19.5546875" customWidth="1"/>
-    <col min="10" max="10" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="37.85546875" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="24.5703125" customWidth="1"/>
+    <col min="8" max="8" width="25.85546875" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" customWidth="1"/>
+    <col min="10" max="10" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">

</xml_diff>